<commit_message>
Switch CZ/SK Six/Eight screen to league-based filtering, bump to top 15
CZ_SK_U23_Six_Eight.xlsx now filters by which Czech/Slovak league file
the player is in (Czech, Czech II, Czech U17, Czech U19, Slovakia,
Slovakia II) instead of passport nationality, matching the treatment
already applied to the Baltics/Scandi/Poland/Slovenia file — so it now
also picks up foreign players in those leagues (e.g. Y. Kambi/Gambia,
Miki García/Spain at Slovak clubs) rather than only CZ/SK passport
holders.

Default top-N raised from 10 to 15 across both screen_six_eight.py and
combine_cz_sk_cms_lamberts.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wzh48iso9dywMF7h3c4ehR
</commit_message>
<xml_diff>
--- a/data/Baltics_Scandi_Poland_Slovenia_U23_Six_Eight.xlsx
+++ b/data/Baltics_Scandi_Poland_Slovenia_U23_Six_Eight.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Baltics + Scandinavia + Finland + Iceland + Poland + Slovenia leagues (by league played in, any nationality)  ·  Top 10 (senior first-team players only)  ·  Progressive passing + defensive-actions volume  ·  Ranked by Six Score</t>
+          <t>Baltics + Scandinavia + Finland + Iceland + Poland + Slovenia leagues (by league played in, any nationality)  ·  Top 15 (senior first-team players only)  ·  Progressive passing + defensive-actions volume  ·  Ranked by Six Score</t>
         </is>
       </c>
     </row>
@@ -1238,6 +1238,329 @@
       </c>
       <c r="Q13" s="5" t="n">
         <v>43.75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>J. Musbaudeen</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Norway II</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>517</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>90.70999999999999</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>73.02</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>65.95999999999999</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>58.06</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>M. Siltanen</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Djurgården</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>885</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>90.58</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>90.31</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>73.33</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>61.54</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>R. Smirnov</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Paide</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>514</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>89.92</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>72.04000000000001</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>68.63</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>A. Doumbia</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Häcken</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v/>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>714</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>89.84</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>84.20999999999999</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>27.27</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>M. Freundlich</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Silkeborg</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>1365</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>400000</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>89.68000000000001</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>89.94</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1698,7 +2021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1714,7 +2037,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Baltics + Scandinavia + Finland + Iceland + Poland + Slovenia leagues (by league played in, any nationality)  ·  Top 10 (senior first-team players only)  ·  Progressive passing, key passes, through passes, shot output  ·  Ranked by Eight Score</t>
+          <t>Baltics + Scandinavia + Finland + Iceland + Poland + Slovenia leagues (by league played in, any nationality)  ·  Top 15 (senior first-team players only)  ·  Progressive passing, key passes, through passes, shot output  ·  Ranked by Eight Score</t>
         </is>
       </c>
     </row>
@@ -2453,6 +2776,329 @@
       </c>
       <c r="Q13" s="5" t="n">
         <v>1.57</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>S. Schierack</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Śląsk Wrocław</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Poland III</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>1489</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>93.98999999999999</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>L. Kolstad</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Eidsvold</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Norway III</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v/>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>575</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>91.73999999999999</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>I. Hjorteseth</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Sotra</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Norway III</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>628</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>90.79000000000001</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>2.29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>A. Przyborek</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>1035</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>90.62</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>J. Bieroński</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Tychy 71</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Poland II</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Senior First Team</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>1508</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>90.52</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>0.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>